<commit_message>
switch the demo clip
</commit_message>
<xml_diff>
--- a/examples/review_demo/results.xlsx
+++ b/examples/review_demo/results.xlsx
@@ -534,7 +534,7 @@
     <row r="2" ht="70" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>examples/part_16_reel.mp4</t>
+          <t>examples/iltalehti_reel.mp4</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -543,35 +543,35 @@
         </is>
       </c>
       <c r="C2" s="2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>["nonstandard_label"]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>[{"name": "thestoryofourhome-pl", "votes": 3}]</t>
+          <t>[{"name": "iltalehti", "votes": 3}]</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>[{"name": "thestoryofourhome-pl", "votes": 3}]</t>
+          <t>[{"name": "iltalehti", "votes": 3}]</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>["thestoryofourhome-pl"]</t>
+          <t>["iltalehti"]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>[{"forward": "thestoryofourhome-pl", "reverse": "thestoryofourhome-pl", "similarity": 1.0}]</t>
+          <t>[{"forward": "iltalehti", "reverse": "iltalehti", "similarity": 1.0}]</t>
         </is>
       </c>
       <c r="I2" s="2" t="n">
-        <v>8.842166666666667</v>
+        <v>50.9</v>
       </c>
       <c r="J2" s="2" t="inlineStr"/>
       <c r="K2" s="2" t="n"/>

</xml_diff>